<commit_message>
solved mate choice data
</commit_message>
<xml_diff>
--- a/data/Mate choice FINAL.xlsx
+++ b/data/Mate choice FINAL.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kigha\Documents\00phdyr1\ALAN\mate choice\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kigha\Documents\00phdyr1\artlight_bio708\artlight\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9372659C-16CC-4D63-A0A1-4ED793773D4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9249BE5B-B27D-40A6-8198-CB2A0B8C9CFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FinalClean" sheetId="2" r:id="rId1"/>
@@ -174,12 +174,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="hh:mm:ss;@"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Verdana"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -274,23 +281,24 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -573,7 +581,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97DC24AB-47C7-4640-B216-A5B2ED1624F0}">
-  <dimension ref="A1:D435"/>
+  <dimension ref="A1:G435"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="6.73046875" style="13" bestFit="1" customWidth="1"/>
@@ -583,7 +591,7 @@
     <col min="5" max="16384" width="9.06640625" style="13"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:7">
       <c r="A1" s="14" t="s">
         <v>21</v>
       </c>
@@ -596,8 +604,9 @@
       <c r="D1" s="14" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="G1" s="15"/>
+    </row>
+    <row r="2" spans="1:7">
       <c r="A2" s="13" t="s">
         <v>15</v>
       </c>
@@ -610,8 +619,9 @@
       <c r="D2" s="13">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
+      <c r="G2" s="15"/>
+    </row>
+    <row r="3" spans="1:7">
       <c r="A3" s="13" t="s">
         <v>15</v>
       </c>
@@ -624,8 +634,9 @@
       <c r="D3" s="13">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:4">
+      <c r="G3" s="15"/>
+    </row>
+    <row r="4" spans="1:7">
       <c r="A4" s="13" t="s">
         <v>15</v>
       </c>
@@ -638,8 +649,9 @@
       <c r="D4" s="13">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:4">
+      <c r="G4" s="15"/>
+    </row>
+    <row r="5" spans="1:7">
       <c r="A5" s="13" t="s">
         <v>15</v>
       </c>
@@ -653,7 +665,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:7">
       <c r="A6" s="13" t="s">
         <v>15</v>
       </c>
@@ -667,7 +679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:7">
       <c r="A7" s="13" t="s">
         <v>15</v>
       </c>
@@ -681,7 +693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:7">
       <c r="A8" s="13" t="s">
         <v>15</v>
       </c>
@@ -695,7 +707,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:7">
       <c r="A9" s="13" t="s">
         <v>15</v>
       </c>
@@ -709,7 +721,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:7">
       <c r="A10" s="13" t="s">
         <v>15</v>
       </c>
@@ -723,7 +735,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:7">
       <c r="A11" s="13" t="s">
         <v>15</v>
       </c>
@@ -737,7 +749,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:7">
       <c r="A12" s="13" t="s">
         <v>15</v>
       </c>
@@ -751,7 +763,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:7">
       <c r="A13" s="13" t="s">
         <v>15</v>
       </c>
@@ -765,7 +777,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:7">
       <c r="A14" s="13" t="s">
         <v>15</v>
       </c>
@@ -779,7 +791,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:7">
       <c r="A15" s="13" t="s">
         <v>15</v>
       </c>
@@ -793,7 +805,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:7">
       <c r="A16" s="13" t="s">
         <v>15</v>
       </c>

</xml_diff>